<commit_message>
revise: adopt Partner review feedback on work plan
Changes:
- Drop AX-A5 standalone (Weihai replicability), merge into AX-A2 → 10 analyses
- Move AX-B1/B2 to Day 1 (Partner executes directly)
- WS-C3 can start Day 2 with preliminary assumptions, finalize Day 3
- Add Case PDF confirmation flag — data may be incomplete in markdown
- Update xlsx to match (merged AX-A2, deleted AX-A5 row)

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/InstantRetail/Tier3-4Strategy/04-work-plan.xlsx
+++ b/InstantRetail/Tier3-4Strategy/04-work-plan.xlsx
@@ -690,7 +690,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -855,12 +855,12 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Three Hemorrhage-Cities Profit Path Analysis</t>
+          <t>Three Hemorrhage-Cities Profit Path + Weihai Model Insights</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>How does each of 3 priority cities (Quanzhou/Huizhou/Weihai) achieve EBIT+? Are paths different?</t>
+          <t>(1) Quanzhou/Huizhou/Weihai EBIT+ paths — same or different? (2) Can Weihai model replicate?</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
@@ -1046,62 +1046,62 @@
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>AX-A5</t>
+          <t>AX-B1</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>WS-A</t>
+          <t>WS-B</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Weihai Model Replicability Assessment</t>
+          <t>Meituan Public Financials Research</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Can Weihai formula be replicated? What are preconditions?</t>
+          <t>What does Meituan spend on subsidies and R&amp;D per order in Tier 3-4?</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>Compare Weihai driver profile vs. other cities; rank by Weihai-fit; AOV uplift pathway</t>
+          <t>Search Meituan 2024 annual report; investor presentations; analyst call transcripts; 四五线城市 subsidy data</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>10-city dataset</t>
+          <t>Meituan IR, Bloomberg, Goldman/DB reports</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>01-problem-definition.md</t>
+          <t>Public financials / analyst reports</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>Available</t>
+          <t>Need (web search)</t>
         </is>
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>Cities ranked by Weihai-fit; AOV uplift pathway</t>
+          <t>Key findings memo: subsidy floor; Tier 3-4 strategy remarks</t>
         </is>
       </c>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>Partially replicable in C7/C1; not in C9/C10 short-term</t>
+          <t>National data only; no city-level; medium confidence</t>
         </is>
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="L6" s="7" t="inlineStr">
         <is>
-          <t>AX-A1, A2 (parallel)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="M6" s="7" t="inlineStr">
@@ -1113,7 +1113,7 @@
     <row r="7" ht="60" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>AX-B1</t>
+          <t>AX-B2</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -1123,27 +1123,27 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Meituan Public Financials Research</t>
+          <t>JD.com Public Financials Research</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>What does Meituan spend on subsidies and R&amp;D per order in Tier 3-4?</t>
+          <t>What is JD.com instant retail strategy in lower-tier cities?</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>Search Meituan 2024 annual report; investor presentations; analyst call transcripts; 四五线城市 subsidy data</t>
+          <t>Search JD.com 2024 annual report; JD到家 investor materials; Analysys market share</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Meituan IR, Bloomberg, Goldman/DB reports</t>
+          <t>JD IR; Analysys; iiMedia</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>Public financials / analyst reports</t>
+          <t>Public financials</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
@@ -1153,12 +1153,12 @@
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>Key findings memo: subsidy floor; Tier 3-4 strategy remarks</t>
+          <t>Key findings memo: competitive intensity; JD到家 differentiation</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>National data only; no city-level; medium confidence</t>
+          <t>Medium confidence</t>
         </is>
       </c>
       <c r="K7" s="7" t="inlineStr">
@@ -1168,7 +1168,7 @@
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>AX-B1 (parallel)</t>
         </is>
       </c>
       <c r="M7" s="7" t="inlineStr">
@@ -1180,7 +1180,7 @@
     <row r="8" ht="60" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>AX-B2</t>
+          <t>AX-B3</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -1190,42 +1190,42 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>JD.com Public Financials Research</t>
+          <t>Competitive Intensity Scenario Analysis</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>What is JD.com instant retail strategy in lower-tier cities?</t>
+          <t>How do competitive scenarios constrain subsidy reduction options?</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Search JD.com 2024 annual report; JD到家 investor materials; Analysys market share</t>
+          <t>Synthesize B1+B2 into 3 scenarios (high/med/low); subsidy floor per scenario; response options</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>JD IR; Analysys; iiMedia</t>
+          <t>AX-B1, B2 outputs</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Public financials</t>
+          <t>B1+B2 research</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>Need (web search)</t>
+          <t>Pending B1/B2</t>
         </is>
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>Key findings memo: competitive intensity; JD到家 differentiation</t>
+          <t>3x3 scenario matrix; subsidy floor per scenario</t>
         </is>
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
-          <t>Medium confidence</t>
+          <t>Even high-competition: some subsidy reduction feasible if targeting low-value users only</t>
         </is>
       </c>
       <c r="K8" s="7" t="inlineStr">
@@ -1235,7 +1235,7 @@
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
-          <t>AX-B1 (parallel)</t>
+          <t>AX-B1, B2 (gating)</t>
         </is>
       </c>
       <c r="M8" s="7" t="inlineStr">
@@ -1247,52 +1247,52 @@
     <row r="9" ht="60" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>AX-B3</t>
+          <t>AX-C1</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>WS-B</t>
+          <t>WS-C</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Competitive Intensity Scenario Analysis</t>
+          <t>Subsidy Efficiency Diagnostic</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>How do competitive scenarios constrain subsidy reduction options?</t>
+          <t>How is 4.2元/order subsidy distributed across city and user quality tiers?</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>Synthesize B1+B2 into 3 scenarios (high/med/low); subsidy floor per scenario; response options</t>
+          <t>Cross-city comparison: subsidy/order vs. high-value user%; worst efficiency cities</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>AX-B1, B2 outputs</t>
+          <t>Subsidy and user% per city</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>B1+B2 research</t>
+          <t>01-problem-definition.md</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>Pending B1/B2</t>
+          <t>Available</t>
         </is>
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
-          <t>3x3 scenario matrix; subsidy floor per scenario</t>
+          <t>Subsidy efficiency ranking table; waste rate proxy</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>Even high-competition: some subsidy reduction feasible if targeting low-value users only</t>
+          <t>C10 has highest subsidy + lowest high-value% = worst efficiency</t>
         </is>
       </c>
       <c r="K9" s="7" t="inlineStr">
@@ -1302,7 +1302,7 @@
       </c>
       <c r="L9" s="7" t="inlineStr">
         <is>
-          <t>AX-B1, B2 (gating)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="M9" s="7" t="inlineStr">
@@ -1314,7 +1314,7 @@
     <row r="10" ht="60" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>AX-C1</t>
+          <t>AX-C2</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
@@ -1324,22 +1324,22 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Subsidy Efficiency Diagnostic</t>
+          <t>High-Value User Improvement Potential Analysis</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>How is 4.2元/order subsidy distributed across city and user quality tiers?</t>
+          <t>What does Weihai (26%) vs. Ganzhou (15%) gap tell us about improvement potential?</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Cross-city comparison: subsidy/order vs. high-value user%; worst efficiency cities</t>
+          <t>Compare Weihai vs. Ganzhou characteristics; identify structural drivers of 11pp gap</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Subsidy and user% per city</t>
+          <t>City and user characteristics; category mix; large super%</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -1349,17 +1349,17 @@
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>Available</t>
+          <t>Partial (断面; no longitudinal)</t>
         </is>
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>Subsidy efficiency ranking table; waste rate proxy</t>
+          <t>Gap decomposition; qualitative improvement pathway</t>
         </is>
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
-          <t>C10 has highest subsidy + lowest high-value% = worst efficiency</t>
+          <t>Gap partly due to category mix + large super depth — both actionable within 12 months</t>
         </is>
       </c>
       <c r="K10" s="7" t="inlineStr">
@@ -1369,7 +1369,7 @@
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>AX-A1 (parallel)</t>
         </is>
       </c>
       <c r="M10" s="7" t="inlineStr">
@@ -1381,7 +1381,7 @@
     <row r="11" ht="60" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>AX-C2</t>
+          <t>AX-C3</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
@@ -1391,42 +1391,42 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>High-Value User Improvement Potential Analysis</t>
+          <t>Subsidy Reallocation Scenario Analysis</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>What does Weihai (26%) vs. Ganzhou (15%) gap tell us about improvement potential?</t>
+          <t>Financial impact of reallocating subsidy from low-value to high-value users?</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>Compare Weihai vs. Ganzhou characteristics; identify structural drivers of 11pp gap</t>
+          <t>3 scenarios (conservative/base/optimistic) for 12-month reallocation; subsidy savings × high-value% trajectory</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>City and user characteristics; category mix; large super%</t>
+          <t>AX-C1, C2 outputs; AX-B3 competitive ceiling</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>01-problem-definition.md</t>
+          <t>AX-C1, C2, B3</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>Partial (断面; no longitudinal)</t>
+          <t>Pending (partial inputs)</t>
         </is>
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>Gap decomposition; qualitative improvement pathway</t>
+          <t>Subsidy savings range per scenario; high-value% trajectory</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>Gap partly due to category mix + large super depth — both actionable within 12 months</t>
+          <t>Conservative: -10% low-value; Base: -20% + retention incentive; Optimistic: full reallocation</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
@@ -1436,7 +1436,7 @@
       </c>
       <c r="L11" s="7" t="inlineStr">
         <is>
-          <t>AX-A1 (parallel)</t>
+          <t>AX-C1, C2, AX-B3 (gating)</t>
         </is>
       </c>
       <c r="M11" s="7" t="inlineStr">
@@ -1445,73 +1445,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="60" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>AX-C3</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>WS-C</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>Subsidy Reallocation Scenario Analysis</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>Financial impact of reallocating subsidy from low-value to high-value users?</t>
-        </is>
-      </c>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t>3 scenarios (conservative/base/optimistic) for 12-month reallocation; subsidy savings × high-value% trajectory</t>
-        </is>
-      </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>AX-C1, C2 outputs; AX-B3 competitive ceiling</t>
-        </is>
-      </c>
-      <c r="G12" s="7" t="inlineStr">
-        <is>
-          <t>AX-C1, C2, B3</t>
-        </is>
-      </c>
-      <c r="H12" s="7" t="inlineStr">
-        <is>
-          <t>Pending (partial inputs)</t>
-        </is>
-      </c>
-      <c r="I12" s="7" t="inlineStr">
-        <is>
-          <t>Subsidy savings range per scenario; high-value% trajectory</t>
-        </is>
-      </c>
-      <c r="J12" s="7" t="inlineStr">
-        <is>
-          <t>Conservative: -10% low-value; Base: -20% + retention incentive; Optimistic: full reallocation</t>
-        </is>
-      </c>
-      <c r="K12" s="7" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="L12" s="7" t="inlineStr">
-        <is>
-          <t>AX-C1, C2, AX-B3 (gating)</t>
-        </is>
-      </c>
-      <c r="M12" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
+    <row r="12" ht="60" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>